<commit_message>
올리브영 수동 데이터 반영 (2026-07-18, 2026-07-19, TOP10)
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-18.xlsx
+++ b/data/daily/2026-07/2026-07-18.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1447,32 +1448,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1485,10 +1486,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -1497,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1532,7 +1533,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1554,7 +1555,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1576,7 +1577,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1598,7 +1599,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1620,7 +1621,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1639,10 +1640,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>26.7</v>
+        <v>27.5</v>
       </c>
       <c r="D9" t="n">
         <v>5</v>
@@ -1651,7 +1652,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1664,7 +1665,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1686,7 +1687,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1705,10 +1706,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D12" t="n">
         <v>5</v>
@@ -1717,7 +1718,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +1728,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>
@@ -1739,8 +1740,322 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[1+1]알디콤 속쓰헤소제 4포입 3종(플러스,에이,브이)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>알디콤</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>15,300원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[7월 올영픽/파격특가] 멜라메이트 구미/로우슈가/버라이어티팩 구미</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>멜라메이트</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>12,900원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>34,010원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[7월 올영픽/1일1정] 바이탈뷰티 메타그린 슬림업 30일 (+15일)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>바이탈뷰티</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>26,900원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[1+1]알디콤 Plus 속쓰헤소제 21ml 4포입</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>알디콤</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>15,300원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[골라담기] CJ웰케어 건강루틴 가격혁명 10종 택1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>멀티비타민/종합비타민</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 14일</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>오쏘몰</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>55,900원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 콜레올로지 컷팅 젤리 레몬/키위/석류 10+2+2포 기획</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>18,400원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 코자아 시목성 멜라토닌 함유 젤리 기획 (+10구미케피드)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>코자아</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>30,900원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[7월 올영픽/서현PICK] 콜레올로지 PRO 600mg*30(+10)/60정 단품</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>17,400원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>